<commit_message>
Rework budget to Q4-2026 stub with explicit assumption cells
2026 is treated as a Q4-only stub (25% of a full year's operating
budget) rather than a full year, per updated guidance. Fundraising is
modeled separately from spending: assumes the full CHF 100-200K target
is raised in 2026 and spent down through 2027-2028 (reserve carried
forward), rather than scaling fundraising by the same quarter-year
fraction as spending.

Both the spending-year-fraction and fundraising-share assumptions are
now explicit, editable cells (highlighted in the spreadsheet) that
every other figure derives from via formula, instead of being baked
into hardcoded numbers - makes it easy to test a different split.
</commit_message>
<xml_diff>
--- a/operations/budget-2026-2028.xlsx
+++ b/operations/budget-2026-2028.xlsx
@@ -44,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E2F3"/>
         <bgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,22 +96,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,10 +476,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -485,21 +490,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Auf — Draft Budget, Years 1–3 (2026–2028)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
+          <t>Auf — Draft Budget, Years 1–3 (Q4 2026 – 2028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status: draft, not approved. Amounts CHF. Years 2027-2028 repeat Year 1's figures as a flat placeholder - no real multi-year plan exists yet (see notes).</t>
+          <t>Status: draft, not approved. Amounts CHF. Yellow cells are the live assumptions — everything else is a formula off them.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SUMMARY</t>
+          <t>ASSUMPTIONS (edit these — everything below follows)</t>
         </is>
       </c>
     </row>
@@ -507,7 +512,7 @@
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -520,137 +525,82 @@
           <t>2028</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>3-yr total</t>
-        </is>
-      </c>
+      <c r="E5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Fundraising target — low</t>
+          <t>Spending basis — share of a full year's operating budget</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>100000</v>
+        <v>0.25</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E6" s="7">
-        <f>SUM(B6:D6)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Fundraising target — high</t>
+          <t>Fundraising basis — share of the CHF 100k-200k target raised this period</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E7" s="7">
-        <f>SUM(B7:D7)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Operating expenses</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>B25</f>
-        <v/>
-      </c>
-      <c r="C8" s="6">
-        <f>C25</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>D25</f>
-        <v/>
-      </c>
-      <c r="E8" s="7">
-        <f>SUM(B8:D8)</f>
-        <v/>
+          <t>Base full-year fundraising target — low</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Net — low case</t>
-        </is>
-      </c>
-      <c r="B9" s="7">
-        <f>B6-B8</f>
-        <v/>
-      </c>
-      <c r="C9" s="7">
-        <f>C6-C8</f>
-        <v/>
-      </c>
-      <c r="D9" s="7">
-        <f>D6-D8</f>
-        <v/>
-      </c>
-      <c r="E9" s="7">
-        <f>SUM(B9:D9)</f>
-        <v/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Base full-year fundraising target — high</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>200000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Net — high case</t>
-        </is>
-      </c>
-      <c r="B10" s="7">
-        <f>B7-B8</f>
-        <v/>
-      </c>
-      <c r="C10" s="7">
-        <f>C7-C8</f>
-        <v/>
-      </c>
-      <c r="D10" s="7">
-        <f>D7-D8</f>
-        <v/>
-      </c>
-      <c r="E10" s="7">
-        <f>SUM(B10:D10)</f>
-        <v/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Base full-year operating budget</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>REVENUE BY YEAR</t>
+          <t>SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
+      <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -663,334 +613,496 @@
           <t>2028</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>3-yr total</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Donations / sponsorships — low</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Flat placeholder — see donors/strategy.md for tiers/segments. Live pipeline tracked via GitHub Issues (donors/pipeline.md).</t>
-        </is>
+          <t>Fundraising raised — low</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>$B$8*B7</f>
+        <v/>
+      </c>
+      <c r="C14" s="8">
+        <f>$B$8*C7</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>$B$8*D7</f>
+        <v/>
+      </c>
+      <c r="E14" s="9">
+        <f>SUM(B14:D14)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Donations / sponsorships — high</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Same caveat — flat placeholder, not a forecast.</t>
-        </is>
+          <t>Fundraising raised — high</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>$B$9*B7</f>
+        <v/>
+      </c>
+      <c r="C15" s="8">
+        <f>$B$9*C7</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>$B$9*D7</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>SUM(B15:D15)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Membership fees</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>TBD — set annually by the General Assembly per statutes Art. 8; likely negligible relative to donations.</t>
-        </is>
+          <t>Operating expenses</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>$B$10*B6</f>
+        <v/>
+      </c>
+      <c r="C16" s="8">
+        <f>$B$10*C6</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>$B$10*D6</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>SUM(B16:D16)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Total revenue — low</t>
-        </is>
-      </c>
-      <c r="B17" s="7">
-        <f>B14+B16</f>
-        <v/>
-      </c>
-      <c r="C17" s="7">
-        <f>C14+C16</f>
-        <v/>
-      </c>
-      <c r="D17" s="7">
-        <f>D14+D16</f>
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Reserve movement — low</t>
+        </is>
+      </c>
+      <c r="B17" s="9">
+        <f>B14-B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="9">
+        <f>C14-C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="9">
+        <f>D14-D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="9">
+        <f>SUM(B17:D17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Total revenue — high</t>
-        </is>
-      </c>
-      <c r="B18" s="7">
-        <f>B15+B16</f>
-        <v/>
-      </c>
-      <c r="C18" s="7">
-        <f>C15+C16</f>
-        <v/>
-      </c>
-      <c r="D18" s="7">
-        <f>D15+D16</f>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Reserve movement — high</t>
+        </is>
+      </c>
+      <c r="B18" s="9">
+        <f>B15-B16</f>
+        <v/>
+      </c>
+      <c r="C18" s="9">
+        <f>C15-C16</f>
+        <v/>
+      </c>
+      <c r="D18" s="9">
+        <f>D15-D16</f>
+        <v/>
+      </c>
+      <c r="E18" s="9">
+        <f>SUM(B18:D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Cumulative reserve, end of period — low</t>
+        </is>
+      </c>
+      <c r="B19" s="9">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C19" s="9">
+        <f>B19+C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="9">
+        <f>C19+D17</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>OPERATING EXPENSES BY YEAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Cumulative reserve, end of period — high</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="C20" s="9">
+        <f>B20+C18</f>
+        <v/>
+      </c>
+      <c r="D20" s="9">
+        <f>C20+D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>REVENUE BY PERIOD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Illustrative 50/50 split of the ~20,000/year figure — TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Office equipment</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>First-year setup costs are usually front-loaded — repeating Year 1's figure in 2027-2028 likely overestimates equipment specifically. Revisit once Year 1 actuals are known.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>Donations / sponsorships — low</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>$B$8*B7</f>
+        <v/>
+      </c>
+      <c r="C24" s="8">
+        <f>$B$8*C7</f>
+        <v/>
+      </c>
+      <c r="D24" s="8">
+        <f>$B$8*D7</f>
+        <v/>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>100% of the low-case target assumed raised in Q4 2026 - see donors/strategy.md for tiers/segments. Live pipeline tracked via GitHub Issues (donors/pipeline.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Donations / sponsorships — high</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>$B$9*B7</f>
+        <v/>
+      </c>
+      <c r="C25" s="8">
+        <f>$B$9*C7</f>
+        <v/>
+      </c>
+      <c r="D25" s="8">
+        <f>$B$9*D7</f>
+        <v/>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Same assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Membership fees</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>TBD - set annually by the General Assembly per statutes Art. 8; likely negligible relative to donations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>OPERATING EXPENSES BY PERIOD</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <f>$B$10*0.5*B6</f>
+        <v/>
+      </c>
+      <c r="C30" s="8">
+        <f>$B$10*0.5*C6</f>
+        <v/>
+      </c>
+      <c r="D30" s="8">
+        <f>$B$10*0.5*D6</f>
+        <v/>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Illustrative 50% share of the operating budget - TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Office equipment</t>
+        </is>
+      </c>
+      <c r="B31" s="8">
+        <f>$B$10*0.5*B6</f>
+        <v/>
+      </c>
+      <c r="C31" s="8">
+        <f>$B$10*0.5*C6</f>
+        <v/>
+      </c>
+      <c r="D31" s="8">
+        <f>$B$10*0.5*D6</f>
+        <v/>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Illustrative 50% share. First-year setup costs are usually front-loaded - revisit once actuals are known.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>Office rent</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Not yet committed — no space secured. Add as a recurring line starting in whichever year a lease is signed, not retroactively across all three.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Not yet committed - no space secured. Add as a recurring line starting in whichever period a lease is signed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="B25" s="7">
-        <f>SUM(B22:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="7">
-        <f>SUM(C22:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="7">
-        <f>SUM(D22:D24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="B33" s="9">
+        <f>SUM(B30:B32)</f>
+        <v/>
+      </c>
+      <c r="C33" s="9">
+        <f>SUM(C30:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="9">
+        <f>SUM(D30:D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>WHAT THIS BUDGET DOES NOT YET COVER</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>• Direct participant support (seed contributions to founders per statutes Art. 2, mentorship stipends, etc.) - NOT sized here, in any year. Cost per participant/track is still TBD in participants/support-offered.md; once set, it becomes its own line - likely the largest cost driver by Year 2 or 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>• Paid staff - statutes assume an honorary/volunteer board (Art. 17); no salaries budgeted in any year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>• Any statutory audit fee, if the GA appoints auditors (statutes Art. 14) - not yet costed for any year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>• Growth or decline in fundraising capacity - Year 1 is a genuine estimate; Years 2-3 are the same number copy-pasted forward, not a forecast.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>• Direct participant support (seed contributions to founders per statutes Art. 2, mentorship stipends, etc.) - NOT sized here, in any period. Once set, it draws directly on the reserve above rather than requiring fresh fundraising, under the current assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>• Paid staff - statutes assume an honorary/volunteer board (Art. 17); no salaries budgeted in any period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>• Any statutory audit fee, if the GA appoints auditors (statutes Art. 14) - not yet costed for any period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>• Whether 'raise it all in 2026, spend it down after' is actually the right fundraising strategy - a clean modeling assumption, not a decided strategy. Change the assumption cells above to test other splits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>OPEN QUESTIONS FOR THE FOUNDING TEAM</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>☐ Confirm whether Years 2-3 should really repeat Year 1's fundraising target, or whether growth/decline assumptions should be modeled instead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>☐ Confirm the events / office-equipment split, and whether equipment costs should be lower in Years 2-3 versus Year 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>☐ Confirm timeline for securing office space and expected rent, and which year it should first appear in.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>☐ Set a cost-per-participant figure in participants/support-offered.md and add it as a budget line, ideally per year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
-        <is>
-          <t>☐ Approve this plan via board resolution and/or GA per operations/finance.md's budget cycle - note the statutes' annual-budget process (Art. 12) is a one-year cycle, so a 3-year plan needs re-approval or re-confirmation annually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>☐ Confirm 'raise ~100% in 2026, live off reserve through 2028' is the intended strategy vs. continuing to fundraise annually (change the Fundraising basis assumption row if not).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>☐ Confirm the events / office-equipment split for Q4 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>☐ Confirm timeline for securing office space and expected rent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>☐ Set a cost-per-participant figure in participants/support-offered.md and add it as a budget line - this is what would actually draw down the reserve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>☐ Approve this plan via board resolution and/or GA per operations/finance.md's budget cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>See operations/budget-2026-2028.md in the auf.so repo for the full narrative version, and operations/finance.md, donors/strategy.md, donors/reporting.md for related process.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Spread fundraising across 2026-2027 instead of a single 2026 raise
Adopts the user's revised assumption cells: 50%/100%/0% of the target
raised in Q4 2026/2027/2028 (low case: 50k then 100k; high case: 100k
then 200k), instead of the previous "raise it all in 2026" model. Also
adopts their trimmed low-case 2028 grant count (6 units instead of 7)
to keep that scenario solvent. Costs are unchanged.

Recalculated finding: the low case now stays solvent through all three
years, but ends 2028 with only ~CHF 4,000 of reserve - essentially
break-even, not a real margin. The high case ends with a much healthier
~CHF 124,000 buffer. Updated the "key finding" framing in both the
markdown and spreadsheet from "negative" to "thin but positive."
</commit_message>
<xml_diff>
--- a/operations/budget-2026-2028.xlsx
+++ b/operations/budget-2026-2028.xlsx
@@ -42,7 +42,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00990000"/>
+      <color rgb="001B5E20"/>
       <sz val="11"/>
     </font>
     <font>
@@ -58,8 +58,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-        <bgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -520,14 +520,14 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>KEY FINDING: LOW-CASE FUNDRAISING TARGET MAY NOT BE ENOUGH</t>
+          <t>UPDATED FINDING: LOW CASE NOW VIABLE, BUT ONLY JUST (+CHF 4,000 BY END OF 2028)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Once beneficiary grants are sized in (per counsel's suggested ramp-up below), the low-case CHF 100,000 fundraising target does NOT cover three years of operations - cumulative reserve goes negative by end of 2028 (~-56,000). The high case (200,000) survives with only a thin ~24,000 buffer left. See 'Reading this plan' notes at the bottom for options.</t>
+          <t>Revised fundraising schedule (raised across Q4 2026 AND 2027, not all at once) plus a trimmed 2028 grant count in the low case keeps the cumulative reserve positive throughout - but only by ~CHF 4,000 at the end of 2028 in the low case. High case ends with a much healthier ~CHF 124,000 buffer. Treat the low case as break-even with no margin for error, not as comfortably solved.</t>
         </is>
       </c>
     </row>
@@ -580,10 +580,10 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="8" t="n">
         <v>1</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0</v>
@@ -622,7 +622,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>BENEFICIARY GRANTS - COUNSEL'S SUGGESTED RAMP-UP (direct inputs per period)</t>
+          <t>BENEFICIARY GRANTS (direct inputs per period)</t>
         </is>
       </c>
     </row>
@@ -663,11 +663,11 @@
         <v>40000</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>70000</v>
+        <v>60000</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Q4 2026 = ~1 unit, my placeholder (counsel didn't size a partial quarter). 2027 = counsel's 'Jahr 1' (4-5 units). 2028 = counsel's 'Jahr 2' (7-8 units).</t>
+          <t>Q4 2026 = ~1 unit placeholder. 2027 = 4 units. 2028 trimmed to 6 units (from 7) to keep the low case solvent under the new revenue schedule.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Same mapping, high end of counsel's per-period range.</t>
+          <t>Unchanged from the previous version.</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Reduced sharply per counsel: without a leased office, only a few electronic devices are needed.</t>
+          <t>Unchanged.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>New line replacing flat CHF 0 rent, which counsel flagged as incoherent next to a high equipment line. Illustrative, based on Impact Hub Zürich public pricing (~215/month Medium, ~55/month Community) - not a real quote.</t>
+          <t>Unchanged - illustrative, not a real quote.</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>New line per counsel's suggestion (Google Workspace or similar) - illustrative, TBD.</t>
+          <t>Unchanged - illustrative.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>100% of the low-case target assumed raised in Q4 2026 - see donors/strategy.md.</t>
+          <t>50% of the low-case target raised in Q4 2026, the rest in 2027 - see donors/strategy.md.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Same assumption.</t>
+          <t>Same schedule, high case.</t>
         </is>
       </c>
     </row>
@@ -1245,35 +1245,35 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>• Whether 'raise it all in 2026, spend it down after' is the right strategy - see the key finding at the top; under this assumption the low case isn't enough once grants are real.</t>
+          <t>• Fundraising in 2028 - this plan assumes no new money is raised in 2028; the low case has almost no room to absorb a shortfall if that's wrong.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>READING THIS PLAN — CLOSING THE LOW-CASE GAP</t>
+          <t>READING THIS PLAN</t>
         </is>
       </c>
     </row>
     <row r="54" ht="26" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>1. Fundraise above CHF 100,000, or target the higher end of the range, if the grant ramp-up is the real plan.</t>
+          <t>The low case now survives all three years, but CHF 4,000 at the end of 2028 is not a buffer, it's a rounding error.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="26" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>2. Slow the grant ramp-up - fewer funded units in 2028, or smaller grants than the CHF 10,000 cap per unit.</t>
+          <t>Anything that pushes cost up or fundraising down even slightly (one more grant, a slower 2027 raise, a lease instead of coworking) puts the low case negative.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="26" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>3. Keep fundraising in 2027 and 2028 instead of a single 2026 raise - change the Fundraising basis assumption row.</t>
+          <t>The high case has real room (~CHF 124,000 by end of 2028) - the more realistic cushion to plan around if fundraising lands anywhere above the low end.</t>
         </is>
       </c>
     </row>
@@ -1287,47 +1287,40 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>☐ Decide how to close the low-case funding gap (raise more, fund fewer beneficiaries, or keep fundraising past 2026).</t>
+          <t>☐ Given how thin the low-case margin is, decide whether 6 funded units in 2028 is a hard cap in that scenario, or whether fundraising should continue into 2028.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>☐ Confirm the Q4 2026 grants estimate (~1 unit, CHF 10,000) - a placeholder, not something counsel sized.</t>
+          <t>☐ Confirm the coworking/SaaS estimates - both are still illustrative guesses, not real quotes.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>☐ Confirm the coworking/SaaS estimates - both are illustrative guesses, not real quotes.</t>
+          <t>☐ Confirm timeline for securing dedicated office space, and when coworking membership would be replaced by a lease.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>☐ Confirm timeline for securing dedicated office space, and when coworking membership would be replaced by a lease.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
           <t>☐ Approve this plan via board resolution and/or GA per operations/finance.md's budget cycle.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
         <is>
           <t>See operations/budget-2026-2028.md in the auf.so repo for the full narrative version, and operations/finance.md, donors/strategy.md, participants/support-offered.md, donors/reporting.md for related process.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="23">
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A56:F56"/>
@@ -1339,19 +1332,18 @@
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A63:F63"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>